<commit_message>
fix: skip phantom COPY_SOURCE_MONTH_SAMPLE rows in source-order writer
- Add COPY_SOURCE_MONTH_SAMPLE and UNKNOWN to GENERATED_FILE_ORDER_POLICIES
  in complete_v1_source_order_writer.py to prevent admin consumable preview
  rows from being preserved during source-order re-layout

Bug fixes:
- 決起コンパ: no longer shows 12 months (was phantom data from old runs)
- トイレットペーパー/手洗い洗剤: no longer duplicated at Row 38-39
  without account code under wrong parent account (5004086291)
- Row 48-49 (Hand wash/Toilet paper) correct with account 5005016372

Also includes:
- Bug #21: skip 配布数 rules in allocator.py
- Requirements doc updates (cai_tien_nhap_du_lieu_chung.md)
- New files: cost_center_context.py, test coverage improvements
</commit_message>
<xml_diff>
--- a/docs/MP2027/source_file_order.xlsx
+++ b/docs/MP2027/source_file_order.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>システム課金金額(Simulation)_FY2027_July.2026 ~ Dec.2026(Change AMS &amp; PLM price).xls</t>
+          <t>システム課金金額(Simulation)_FY2027_Jan.2027 ~ March.2027(Change SAP price).xls</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>IT simulation Jul-Dec source</t>
+          <t>IT simulation source</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>システム課金金額(Simulation)_FY2027_Jan.2027 ~ March.2027(Change SAP price).xls</t>
+          <t>システム課金金額(Simulation)_FY2027_July.2026 ~ Dec.2026(Change AMS &amp; PLM price).xls</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -581,7 +581,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>IT simulation Jan-Mar source</t>
+          <t>IT simulation source</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: export FORM dynamically by source order
</commit_message>
<xml_diff>
--- a/docs/MP2027/source_file_order.xlsx
+++ b/docs/MP2027/source_file_order.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -449,6 +449,16 @@
           <t>description</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>period_start</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>period_end</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -530,6 +540,16 @@
           <t>IT simulation Apr-Jun source</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>202604</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>202606</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -557,6 +577,16 @@
           <t>IT simulation source</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>202701</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>202703</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -582,6 +612,16 @@
       <c r="E6" t="inlineStr">
         <is>
           <t>IT simulation source</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>202612</t>
         </is>
       </c>
     </row>

</xml_diff>